<commit_message>
med vo 26 data
</commit_message>
<xml_diff>
--- a/golf_streamlit/data/baneinfo.xlsx
+++ b/golf_streamlit/data/baneinfo.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\c624kh1\Documents\My Projects\min_git\golf_streamlit\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF387D10-4003-41A6-8813-F323D9C41665}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{301F5554-18BD-4DD4-8DC1-B92678A83B77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2304" yWindow="2304" windowWidth="13044" windowHeight="11484" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="24">
   <si>
     <t>Bane</t>
   </si>
@@ -89,6 +89,9 @@
   </si>
   <si>
     <t>CH</t>
+  </si>
+  <si>
+    <t>The Club at Olde Stone</t>
   </si>
 </sst>
 </file>
@@ -456,7 +459,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="24.33203125" customWidth="1"/>
@@ -672,6 +675,20 @@
         <v>18</v>
       </c>
       <c r="D15">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>23</v>
+      </c>
+      <c r="B16" t="s">
+        <v>20</v>
+      </c>
+      <c r="C16">
+        <v>18</v>
+      </c>
+      <c r="D16">
         <v>72</v>
       </c>
     </row>

</xml_diff>